<commit_message>
🔄 Atualização 2026-07-01 20:51
</commit_message>
<xml_diff>
--- a/Constantine_WhatsApp_Validado.xlsx
+++ b/Constantine_WhatsApp_Validado.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -70,7 +67,7 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -438,14 +435,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -466,12 +464,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Melhor Número</t>
+          <t>WhatsApp 1</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Todos os Números</t>
+          <t>WhatsApp 2</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>WhatsApp 3</t>
         </is>
       </c>
     </row>
@@ -496,11 +499,8 @@
           <t>+5544999723481</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>+5544999723481 (✅) | +5544999723483 (❌)</t>
-        </is>
-      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -518,16 +518,9 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>+5542999053336</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>+5542999053336 (❌)</t>
-        </is>
-      </c>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -550,11 +543,8 @@
           <t>+5544999731590</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>+5544999731590 (✅) | +5544910054586 (❌)</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -572,16 +562,9 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>+5544999703018</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>+5544999703018 (❌) | +5544991078706 (❌)</t>
-        </is>
-      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -599,16 +582,9 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>+5544999418887</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>+5544999418887 (❌) | +5544991449979 (❌)</t>
-        </is>
-      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -633,9 +609,10 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>+5544991666320 (❌) | +5544991671110 (✅) | +5544991661591 (❌)</t>
-        </is>
-      </c>
+          <t>+5544991661591</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -660,9 +637,10 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>+5511982099902 (✅) | +5511964688864 (✅)</t>
-        </is>
-      </c>
+          <t>+5511964688864</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -687,9 +665,10 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>+5544991090818 (✅) | +5544999105888 (✅) | +5544999385888 (✅)</t>
-        </is>
-      </c>
+          <t>+5544999105888</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -709,14 +688,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>+5543988139457</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>+5543999761999</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>+5543988139457 (❌) | +5543999761999 (✅)</t>
-        </is>
-      </c>
+      <c r="F10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -739,38 +719,32 @@
           <t>+5566999853662</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>+5566999853662 (✅) | +5544998171111 (✅)</t>
-        </is>
-      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>1001</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>JOSE SUSUMU SAKAMOTO</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>+5544999918000</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>+5544999918000 (❌) | +5544988480000 (❌)</t>
-        </is>
-      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -793,11 +767,8 @@
           <t>+5544991260944</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>+5544991260944 (✅) | +5544999640092 (❌)</t>
-        </is>
-      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -820,38 +791,32 @@
           <t>+5544984172062</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>+5544984172062 (✅) | +5544998365292 (✅) | +5544984531646 (❌)</t>
-        </is>
-      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>1004</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>CRISTINA GIATTI MARQUES DE SOUZA</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>+5544999161629</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>+5544999161629 (❌)</t>
-        </is>
-      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -871,41 +836,35 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>+5544999613958</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>+5544999613958 (✅) | +5544991022332 (❌)</t>
-        </is>
-      </c>
+          <t>+5544991022332</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>1103</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>ANDERSON CLAYTON GOMES</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>+5544999221399</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>+5544999221399 (❌) | +5544984849933 (❌)</t>
-        </is>
-      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -928,11 +887,8 @@
           <t>+5544991135342</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>+5544991135342 (✅) | +5544910071004 (❌)</t>
-        </is>
-      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -957,9 +913,10 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>+5544991140030 (✅) | +5544999736453 (✅)</t>
-        </is>
-      </c>
+          <t>+5544999736453</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -979,14 +936,11 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>+5544999564100</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>+5544999564100 (✅) | +5544998070303 (❌)</t>
-        </is>
-      </c>
+          <t>+5544998070303</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1006,14 +960,11 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>+5544998079406</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>+5544998079406 (✅) | +5544998070010 (✅)</t>
-        </is>
-      </c>
+          <t>+5544998070010</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1031,16 +982,9 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>+5544991174040</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>+5544991174040 (❌) | +5544991489622 (❌)</t>
-        </is>
-      </c>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1063,11 +1007,8 @@
           <t>+5544999914534</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>+5544999914534 (✅) | +5544991074534 (❌)</t>
-        </is>
-      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1085,16 +1026,9 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>+5544991191898</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>+5544991191898 (❌) | +5544991174044 (❌)</t>
-        </is>
-      </c>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1119,9 +1053,10 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>+5544991580503 (✅) | +5544991050825 (✅)</t>
-        </is>
-      </c>
+          <t>+5544991050825</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1144,11 +1079,8 @@
           <t>+5544999690541</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>+5544999695501 (❌) | +5544999690541 (✅)</t>
-        </is>
-      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1171,11 +1103,8 @@
           <t>+5544999855030</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>+5544999855030 (✅) | +5544998550103 (✅)</t>
-        </is>
-      </c>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1198,11 +1127,8 @@
           <t>+5544999639060</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>+5544999639060 (✅) | +5544999639061 (✅)</t>
-        </is>
-      </c>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1220,70 +1146,57 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>+5544999809977</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>+5544999809977 (❌) | +5544999932988 (❌)</t>
-        </is>
-      </c>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>1501</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>JULIENY CRISTINA PEREIRA LOPES PAULINO</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>+5544998181808</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>+5544998181806</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>1502</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>ANDREA PARRA MANREZA CARVALHO</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>+5544998181808</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>+5544998181808 (❌) | +5544998181806 (❌)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>1502</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>ANDREA PARRA MANREZA CARVALHO</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>+5544991482590</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>+5544991482590 (✅) | +5544991061040 (❌)</t>
-        </is>
-      </c>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1306,11 +1219,8 @@
           <t>+5544991188814</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>+5544991188814 (✅)</t>
-        </is>
-      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1328,70 +1238,57 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>+5544999903484</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>+5544999903484 (❌) | +5544998365555 (❌)</t>
-        </is>
-      </c>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>1601</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>POLYANE ALVES LIMA YOKOTA</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>+5544999464012</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>+5544999464012 (❌) | +5544997088972 (❌)</t>
-        </is>
-      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>1602</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>MARIA TEREZA RAMOS TRENTINI</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>+5544991501226</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>+5544991501226 (❌) | +5544999550049 (❌)</t>
-        </is>
-      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>+5544999550049</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1414,11 +1311,8 @@
           <t>+5544999012049</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>+5544999012049 (✅) | +5544991432049 (❌)</t>
-        </is>
-      </c>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -1436,16 +1330,9 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>+5544991475200</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>+5544991475200 (❌) | +5544991275200 (❌)</t>
-        </is>
-      </c>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -1463,70 +1350,57 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>+5544991174040</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>+5544991174040 (❌) | +5544991489622 (❌)</t>
-        </is>
-      </c>
+      <c r="D38" s="3" t="inlineStr"/>
+      <c r="E38" s="3" t="inlineStr"/>
+      <c r="F38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>1702</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>TAQUECO YAMAMOTO</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>+5544999719971</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>+5544999719971 (✅) | +5544998560512 (❌)</t>
-        </is>
-      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>1703</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>PRISCILA AKEMI MANABE SATO</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>+5544991111434</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>+5544991111434 (❌) | +5544998316698 (❌)</t>
-        </is>
-      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>+5544998316698</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -1544,16 +1418,9 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>+5544991777447</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>+5544991777447 (❌) | +5544999067101 (❌)</t>
-        </is>
-      </c>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1573,14 +1440,11 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>+5544991113020</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>+5544991113020 (✅) | +5544999744884 (✅)</t>
-        </is>
-      </c>
+          <t>+5544999744884</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -1598,16 +1462,9 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>+5544998036040</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>+5544998036040 (❌) | +5544999634840 (❌)</t>
-        </is>
-      </c>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1630,11 +1487,8 @@
           <t>+5544999920066</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>+5544999920066 (✅) | +5544984324840 (❌)</t>
-        </is>
-      </c>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1659,9 +1513,10 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>+5544999659044 (✅) | +5544999659041 (✅)</t>
-        </is>
-      </c>
+          <t>+5544999659041</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -1679,16 +1534,9 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>+5544991475200</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>+5544991475200 (❌) | +5544991275200 (❌)</t>
-        </is>
-      </c>
+      <c r="D46" s="3" t="inlineStr"/>
+      <c r="E46" s="3" t="inlineStr"/>
+      <c r="F46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1708,14 +1556,11 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>+5544991045057</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>+5544998279146 (❌) | +5544991045057 (✅)</t>
-        </is>
-      </c>
+          <t>+5544998279146</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1738,11 +1583,8 @@
           <t>+5544998168832</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>+5544998168832 (✅) | +5544999201001 (❌)</t>
-        </is>
-      </c>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -1760,16 +1602,9 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>+5544991495050</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>+5544991495050 (❌) | +5544998344442 (❌)</t>
-        </is>
-      </c>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1792,11 +1627,8 @@
           <t>+5544999751900</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>+5544999751900 (✅) | +5544999751955 (✅)</t>
-        </is>
-      </c>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1819,11 +1651,8 @@
           <t>+5544991395558</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>+5544991728848 (❌) | +5544991395558 (✅)</t>
-        </is>
-      </c>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1843,14 +1672,15 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
+          <t>+5544991113020</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
           <t>+5544999744884</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>+5544991113020 (❌) | +5544999744884 (✅)</t>
-        </is>
-      </c>
+      <c r="F52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1875,9 +1705,10 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>+5544999674012 (✅) | +5544999640623 (✅)</t>
-        </is>
-      </c>
+          <t>+5544999640623</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1897,14 +1728,11 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>+5544991722345</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>+5544998367765 (❌) | +5544991722345 (✅)</t>
-        </is>
-      </c>
+          <t>+5544998367765</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1929,7 +1757,12 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>+5544991727549 (✅) | +5544991583028 (❌) | +5544991182733 (✅)</t>
+          <t>+5544991583028</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>+5544991182733</t>
         </is>
       </c>
     </row>
@@ -1954,38 +1787,32 @@
           <t>+5544991537335</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>+5544991537335 (✅) | +5561999828015 (❌)</t>
-        </is>
-      </c>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>2401</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>JOAO EDSON CHAVENCO</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>+5544999848451</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>+5544999848451 (❌)</t>
-        </is>
-      </c>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>